<commit_message>
Excely: list Vysvětlivky (sloupce, fáze, druhy kapitálu, typy) a komentáře u záhlaví; kontrola zachovává už zadané odpovědi; uloženy první ruční verdikty
</commit_message>
<xml_diff>
--- a/data/Databaze_investoru.xlsx
+++ b/data/Databaze_investoru.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investoři" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vyřazení" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jak číst" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vysvětlivky" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vyřazení" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jak číst" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +39,14 @@
     <font>
       <i val="1"/>
       <color rgb="00999999"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="4">
@@ -70,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -93,6 +102,9 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -167,6 +179,58 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>investor-db</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Název investora. Klik otevře jeho web.
+Příklad: Credo Ventures</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Druh investora, tabulka typů je v listu Vysvětlivky.
+Příklad: VC fond, private equity, anděl</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>V jakých oborech investor investuje (podle toho, co sám deklaruje).
+Příklad: AI, fintech, zdraví; „bez omezení oboru“ = investuje do čehokoli</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>V jakém stadiu vývoje jsou firmy, do kterých investuje — tabulka fází je v listu Vysvětlivky.
+Příklad: pre-seed, seed = velmi mladé firmy</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Kolik obvykle vloží do jedné firmy (tzv. tiket).
+Příklad: 250 tis. – 1 mil. EUR</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Kolik peněz má investor celkem; v závorce co číslo znamená (tabulka v listu Vysvětlivky).
+Příklad: 75,9 mil. EUR (poslední fond)</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Poslední veřejně doložená investice za poslední 3 roky. Klik otevře článek nebo tiskovou zprávu.
+Příklad: Modeinspect (15. 1. 2026)</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2324,10 +2388,548 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId222"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Vysvětlivky</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Co znamená který sloupec</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Sloupec</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Co znamená</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Příklad</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Název investora. Klik otevře jeho web.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Credo Ventures</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Druh investora, tabulka typů je v listu Vysvětlivky.</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>VC fond, private equity, anděl</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Sektor</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>V jakých oborech investor investuje (podle toho, co sám deklaruje).</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>AI, fintech, zdraví; „bez omezení oboru“ = investuje do čehokoli</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Do čeho investuje (fáze)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>V jakém stadiu vývoje jsou firmy, do kterých investuje — tabulka fází je v listu Vysvětlivky.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>pre-seed, seed = velmi mladé firmy</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Typická výše investice</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Kolik obvykle vloží do jedné firmy (tzv. tiket).</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>250 tis. – 1 mil. EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Celkový kapitál</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Kolik peněz má investor celkem; v závorce co číslo znamená (tabulka v listu Vysvětlivky).</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>75,9 mil. EUR (poslední fond)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Doklad, že investuje (firma, datum)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Poslední veřejně doložená investice za poslední 3 roky. Klik otevře článek nebo tiskovou zprávu.</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Modeinspect (15. 1. 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Fáze — v jakém stadiu jsou firmy, do kterých investor investuje</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Fáze</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Co to znamená</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Typická investice</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>pre-seed</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>jen nápad nebo první prototyp, často ještě bez firmy</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>desítky až stovky tisíc EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>první produkt, první zákazníci</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>stovky tisíc až ~2 mil. EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>série A</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>produkt funguje, firma roste a potřebuje peníze na škálování</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>jednotky milionů EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>série B+</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>další růstová kola, expanze do zahraničí</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>desítky milionů EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>růstová fáze</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>zavedená firma, investor kupuje menšinový podíl</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>desítky milionů EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>buyout</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>investor kupuje celou firmu nebo většinu (typické pro private equity)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>desítky až stovky mil. EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Celkový kapitál — co znamená údaj v závorce</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>V závorce</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Co číslo znamená</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>poslední fond</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>velikost posledního uzavřeného fondu</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>cíl fondu</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>kolik fond chce vybrat — uzavření zatím není doložené</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>předchozí fond</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>velikost staršího fondu (aktuální není veřejná)</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>součet fondů</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>všechny fondy investora dohromady</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>spravovaná aktiva</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>vše, co investor spravuje (AUM), i mimo startupy</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>hodnota portfolia</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>současná hodnota firem, ve kterých má podíl — ne volné peníze</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>vlastní kapitál</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>investor investuje vlastní peníze (bez cizích investorů)</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>aktiva celé skupiny</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>majetek celé skupiny vč. nemovitostí — ne jen peníze na investice</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>Typy investorů</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Co to je</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>VC fond</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>fond rizikového kapitálu, investuje do startupů</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>private equity</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>kupuje podíly nebo celé zralé firmy</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>korporátní VC</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>investiční rameno firmy nebo banky</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>family office</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>spravuje a investuje majetek jedné rodiny (a tak se sám označuje)</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>soukromý investor</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>investiční skupina podnikatele, investuje vlastní peníze</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>anděl</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>fyzická osoba investující vlastní peníze do startupů</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>andělský syndikát</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>skupina andělů investující přes společnou firmu</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>„neuvedeno“ = investor údaj veřejně neuvádí; neodhadujeme ho. Částky v jiných měnách jsou přepočtené na EUR kurzem ECB k datu zdroje.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2839,13 +3441,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2861,33 +3463,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>„neuvedeno“ = investor údaj veřejně neuvádí. Neodhadujeme ho.</t>
+          <t>Co znamená který sloupec, fáze (pre-seed, seed…) a údaje u kapitálu: list „Vysvětlivky“ (nebo najeď myší na záhlaví sloupce).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Částky v jiných měnách přepočteny na EUR kurzem ECB k datu zdroje.</t>
+          <t>„neuvedeno“ = investor údaj veřejně neuvádí. Neodhadujeme ho.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Celkový kapitál: v závorce, co číslo znamená (poslední fond / cíl fondu / spravovaná aktiva…).</t>
+          <t>Částky v jiných měnách přepočteny na EUR kurzem ECB k datu zdroje.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Doklad: poslední veřejně doložená investice za poslední 3 roky; klik otevře článek nebo tiskovou zprávu.</t>
+          <t>Celkový kapitál: v závorce, co číslo znamená (poslední fond / cíl fondu / spravovaná aktiva…).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>Doklad: poslední veřejně doložená investice za poslední 3 roky; klik otevře článek nebo tiskovou zprávu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Pravidla zařazení: PLAN.md. Plné záznamy s citacemi: data/records/.</t>
         </is>

</xml_diff>

<commit_message>
Ruční kontrola – vzorek 2 (čistý, kola 2–3): 20 sedí, 2 nesedí, 1 chyběl (91 %); oba vzorky 49/51 = 96 %; věcná shoda slepého AI ověřovatele 86 %; opravy Flying Founders a Hlavenka; import pozná hodnotu vepsanou člověkem
</commit_message>
<xml_diff>
--- a/data/Databaze_investoru.xlsx
+++ b/data/Databaze_investoru.xlsx
@@ -885,7 +885,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>růstová fáze</t>
+          <t>růstová fáze, buyout</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1174,9 +1174,9 @@
           <t>anděl</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>neuvedeno</t>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>B2B software, AI</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2250,142 +2250,143 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId223"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>